<commit_message>
feat: hapus kepribadian (BFI-10) dari kuesioner dan skor KBF
Atas masukan dosen pembimbing. Bobot dibagi ke RIASEC, minat bidang, dan
kesiapan; skema lama tetap ada sebagai pembanding di evaluasi. Uji A.9
menunjukkan penghapusan tidak menurunkan ketepatan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/validasi/lembar_validitas_isi.xlsx
+++ b/docs/validasi/lembar_validitas_isi.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -455,7 +455,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Lembar 'Penilaian' berisi butir kuesioner yang dipakai sistem untuk mengukur minat dan kepribadian.</t>
+          <t>Lembar 'Penilaian' berisi butir kuesioner yang dipakai sistem untuk mengukur minat.</t>
         </is>
       </c>
     </row>
@@ -507,36 +507,29 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Butir minat dijawab responden dengan skala 'sangat tidak suka' sampai 'sangat suka';</t>
+          <t>Seluruh butir dijawab responden dengan skala 'sangat tidak suka' sampai 'sangat suka'.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>butir kepribadian dengan 'sangat tidak setuju' sampai 'sangat setuju'.</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Nama ahli:</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Nama ahli:</t>
+          <t>Bidang keahlian:</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Bidang keahlian:</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Instansi:</t>
         </is>
@@ -553,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1055,22 +1048,22 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>BD_WEB</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Extraversion: kecenderungan bersosialisasi dan energik — butir berarah terbalik</t>
+          <t>Minat pada bidang kerja: Pengembangan web</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang pendiam dan cenderung menahan diri.</t>
+          <t>Membangun situs dan aplikasi web, dari tampilan sampai server.</t>
         </is>
       </c>
       <c r="E20" s="4" t="n"/>
@@ -1080,22 +1073,22 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>BD_MOBILE</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Agreeableness: keramahan, kepercayaan, dan kerja sama</t>
+          <t>Minat pada bidang kerja: Pengembangan mobile</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang mudah percaya kepada orang lain.</t>
+          <t>Membangun aplikasi untuk ponsel Android atau iOS.</t>
         </is>
       </c>
       <c r="E21" s="4" t="n"/>
@@ -1105,22 +1098,22 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>BD_DATA</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Conscientiousness: keteraturan, ketekunan, dan tanggung jawab — butir berarah terbalik</t>
+          <t>Minat pada bidang kerja: Data &amp; analitik</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang cenderung malas.</t>
+          <t>Mengolah dan menganalisis data untuk menjawab pertanyaan bisnis.</t>
         </is>
       </c>
       <c r="E22" s="4" t="n"/>
@@ -1130,22 +1123,22 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>BD_AI</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Neuroticism: kecenderungan cemas dan mudah tertekan — butir berarah terbalik</t>
+          <t>Minat pada bidang kerja: Kecerdasan buatan</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang santai dan bisa menghadapi tekanan dengan baik.</t>
+          <t>Melatih model machine learning atau membangun aplikasi berbasis AI.</t>
         </is>
       </c>
       <c r="E23" s="4" t="n"/>
@@ -1155,22 +1148,22 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>BD_INFRA</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Openness: keterbukaan terhadap pengalaman, imajinasi, dan seni — butir berarah terbalik</t>
+          <t>Minat pada bidang kerja: Infrastruktur &amp; cloud</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang kurang tertarik pada hal-hal yang berbau seni.</t>
+          <t>Mengelola server, cloud, dan otomasi supaya aplikasi tetap berjalan.</t>
         </is>
       </c>
       <c r="E24" s="4" t="n"/>
@@ -1180,22 +1173,22 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>BD_JARINGAN</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Extraversion: kecenderungan bersosialisasi dan energik</t>
+          <t>Minat pada bidang kerja: Jaringan &amp; dukungan TI</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang mudah bergaul dan suka bersosialisasi.</t>
+          <t>Memasang jaringan, merawat perangkat, dan membantu pengguna yang bermasalah.</t>
         </is>
       </c>
       <c r="E25" s="4" t="n"/>
@@ -1205,22 +1198,22 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>BD_KEAMANAN</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Agreeableness: keramahan, kepercayaan, dan kerja sama — butir berarah terbalik</t>
+          <t>Minat pada bidang kerja: Keamanan siber</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang cenderung mencari-cari kesalahan orang lain.</t>
+          <t>Mencari celah keamanan dan melindungi sistem dari serangan.</t>
         </is>
       </c>
       <c r="E26" s="4" t="n"/>
@@ -1230,22 +1223,22 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>BD_DESAIN</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Conscientiousness: keteraturan, ketekunan, dan tanggung jawab</t>
+          <t>Minat pada bidang kerja: Desain UI/UX</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang mengerjakan tugas sampai tuntas dan teliti.</t>
+          <t>Merancang tampilan dan alur aplikasi supaya mudah dipakai.</t>
         </is>
       </c>
       <c r="E27" s="4" t="n"/>
@@ -1255,22 +1248,22 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>BD_MANAJEMEN</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Neuroticism: kecenderungan cemas dan mudah tertekan</t>
+          <t>Minat pada bidang kerja: Manajemen produk &amp; proyek</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang mudah merasa gugup atau cemas.</t>
+          <t>Mengatur prioritas, jadwal, dan orang supaya sebuah produk selesai.</t>
         </is>
       </c>
       <c r="E28" s="4" t="n"/>
@@ -1280,22 +1273,22 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>BD_BISNIS</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Kepribadian (BFI-10)</t>
+          <t>Minat bidang TI</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Openness: keterbukaan terhadap pengalaman, imajinasi, dan seni</t>
+          <t>Minat pada bidang kerja: Analisis bisnis &amp; sistem perusahaan</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Saya melihat diri saya sebagai seseorang yang punya imajinasi yang aktif.</t>
+          <t>Memahami proses bisnis lalu merancang atau menerapkan sistem untuknya.</t>
         </is>
       </c>
       <c r="E29" s="4" t="n"/>
@@ -1305,7 +1298,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>BD_WEB</t>
+          <t>BD_PEMASARAN</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1315,12 +1308,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Pengembangan web</t>
+          <t>Minat pada bidang kerja: Pemasaran digital</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Membangun situs dan aplikasi web, dari tampilan sampai server.</t>
+          <t>Menjalankan dan mengukur kampanye pemasaran di internet.</t>
         </is>
       </c>
       <c r="E30" s="4" t="n"/>
@@ -1330,7 +1323,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>BD_MOBILE</t>
+          <t>BD_GIM</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1340,12 +1333,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Pengembangan mobile</t>
+          <t>Minat pada bidang kerja: Pengembangan gim</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Membangun aplikasi untuk ponsel Android atau iOS.</t>
+          <t>Membuat gim: mekanika, grafis, dan cerita.</t>
         </is>
       </c>
       <c r="E31" s="4" t="n"/>
@@ -1355,7 +1348,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>BD_DATA</t>
+          <t>BD_PERANGKAT</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1365,12 +1358,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Data &amp; analitik</t>
+          <t>Minat pada bidang kerja: Perangkat keras &amp; IoT</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Mengolah dan menganalisis data untuk menjawab pertanyaan bisnis.</t>
+          <t>Memprogram mikrokontroler, sensor, dan perangkat terhubung.</t>
         </is>
       </c>
       <c r="E32" s="4" t="n"/>
@@ -1380,7 +1373,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>BD_AI</t>
+          <t>BD_KUALITAS</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1390,12 +1383,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Kecerdasan buatan</t>
+          <t>Minat pada bidang kerja: Pengujian perangkat lunak</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Melatih model machine learning atau membangun aplikasi berbasis AI.</t>
+          <t>Menguji aplikasi sampai ketemu bug sebelum dipakai orang.</t>
         </is>
       </c>
       <c r="E33" s="4" t="n"/>
@@ -1405,7 +1398,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>BD_INFRA</t>
+          <t>BD_DOKUMENTASI</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1415,12 +1408,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Infrastruktur &amp; cloud</t>
+          <t>Minat pada bidang kerja: Penulisan teknis</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Mengelola server, cloud, dan otomasi supaya aplikasi tetap berjalan.</t>
+          <t>Menulis panduan dan dokumentasi supaya hal teknis mudah dipahami.</t>
         </is>
       </c>
       <c r="E34" s="4" t="n"/>
@@ -1430,7 +1423,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>BD_JARINGAN</t>
+          <t>BD_WEB3</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1440,271 +1433,21 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Minat pada bidang kerja: Jaringan &amp; dukungan TI</t>
+          <t>Minat pada bidang kerja: Blockchain</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Memasang jaringan, merawat perangkat, dan membantu pengguna yang bermasalah.</t>
+          <t>Membangun smart contract dan aplikasi terdesentralisasi.</t>
         </is>
       </c>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>BD_KEAMANAN</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Keamanan siber</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Mencari celah keamanan dan melindungi sistem dari serangan.</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>BD_DESAIN</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Desain UI/UX</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Merancang tampilan dan alur aplikasi supaya mudah dipakai.</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>BD_MANAJEMEN</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Manajemen produk &amp; proyek</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Mengatur prioritas, jadwal, dan orang supaya sebuah produk selesai.</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>BD_BISNIS</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Analisis bisnis &amp; sistem perusahaan</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Memahami proses bisnis lalu merancang atau menerapkan sistem untuknya.</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>BD_PEMASARAN</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Pemasaran digital</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Menjalankan dan mengukur kampanye pemasaran di internet.</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>BD_GIM</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Pengembangan gim</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Membuat gim: mekanika, grafis, dan cerita.</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>BD_PERANGKAT</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Perangkat keras &amp; IoT</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Memprogram mikrokontroler, sensor, dan perangkat terhubung.</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>BD_KUALITAS</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Pengujian perangkat lunak</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Menguji aplikasi sampai ketemu bug sebelum dipakai orang.</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>BD_DOKUMENTASI</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Penulisan teknis</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Menulis panduan dan dokumentasi supaya hal teknis mudah dipahami.</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>BD_WEB3</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Minat bidang TI</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Minat pada bidang kerja: Blockchain</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Membangun smart contract dan aplikasi terdesentralisasi.</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="E2:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>

</xml_diff>